<commit_message>
feat: dia 5 adiciones
</commit_message>
<xml_diff>
--- a/CURSO PHYTON.xlsx
+++ b/CURSO PHYTON.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PHYTON\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F7CEE26-BF57-4640-9CC7-AF800D9B8AAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0A57DC3-F15D-4152-8C43-8D14750AB22E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{7CA30C3A-7750-4E3E-BF5C-BA751071D61C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{7CA30C3A-7750-4E3E-BF5C-BA751071D61C}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="156">
   <si>
     <t>DINAMICO</t>
   </si>
@@ -506,6 +506,12 @@
   </si>
   <si>
     <t>CLASE 20 JUNIO 2026</t>
+  </si>
+  <si>
+    <t>SIEMPRE DEVUELVE TEXTO ASI LE INGRESMOS NUMEROS</t>
+  </si>
+  <si>
+    <t>2:47:02 EJERCICIOS PRACTICOS 1</t>
   </si>
 </sst>
 </file>
@@ -1179,7 +1185,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7891ECEF-2D58-4393-AA3B-41D4700FB936}">
-  <dimension ref="A1:G191"/>
+  <dimension ref="A1:G194"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="4.33203125" customWidth="1"/>
@@ -1877,6 +1883,16 @@
     <row r="191" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B191" t="s">
         <v>137</v>
+      </c>
+    </row>
+    <row r="192" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="C192" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="194" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B194" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>